<commit_message>
Update UI roles and chat history flows
</commit_message>
<xml_diff>
--- a/UI-UX/docs/ui-v1-tz-compliance-checklist-2026-04-30.xlsx
+++ b/UI-UX/docs/ui-v1-tz-compliance-checklist-2026-04-30.xlsx
@@ -255,7 +255,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -315,6 +315,63 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -704,1383 +761,1427 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
     <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>Чек-лист соответствия UI v1 требованиям ТЗ</t>
         </is>
       </c>
-      <c r="B1" s="19" t="n"/>
-      <c r="C1" s="19" t="n"/>
-      <c r="D1" s="19" t="n"/>
-      <c r="E1" s="19" t="n"/>
-      <c r="F1" s="19" t="n"/>
-      <c r="G1" s="19" t="n"/>
-      <c r="H1" s="19" t="n"/>
-      <c r="I1" s="19" t="n"/>
-      <c r="J1" s="19" t="n"/>
-      <c r="K1" s="20" t="n"/>
+      <c r="B1" s="24" t="n"/>
+      <c r="C1" s="24" t="n"/>
+      <c r="D1" s="24" t="n"/>
+      <c r="E1" s="24" t="n"/>
+      <c r="F1" s="24" t="n"/>
+      <c r="G1" s="24" t="n"/>
+      <c r="H1" s="24" t="n"/>
+      <c r="I1" s="24" t="n"/>
+      <c r="J1" s="24" t="n"/>
+      <c r="K1" s="25" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Версия проверки: 2026-04-30. Статус «при наличии backend» означает, что сценарий и экран в UI готовы, но фактические данные, сохранение и метрики должны приходить с серверной части.</t>
-        </is>
-      </c>
-      <c r="B2" s="21" t="n"/>
-      <c r="C2" s="21" t="n"/>
-      <c r="D2" s="21" t="n"/>
-      <c r="E2" s="21" t="n"/>
-      <c r="F2" s="21" t="n"/>
-      <c r="G2" s="21" t="n"/>
-      <c r="H2" s="21" t="n"/>
-      <c r="I2" s="21" t="n"/>
-      <c r="J2" s="21" t="n"/>
-      <c r="K2" s="22" t="n"/>
-    </row>
-    <row r="3"/>
+          <t>Версия проверки: 2026-05-05. Статус «при наличии backend» означает, что сценарий и экран в UI готовы, но фактические данные, сохранение и метрики должны приходить с серверной части. Учтены ответы заказчика от 05.05.2026 по ролям, авторизации, истории диалогов, поиску по чатам и расчетному модулю.</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="n"/>
+      <c r="C2" s="26" t="n"/>
+      <c r="D2" s="26" t="n"/>
+      <c r="E2" s="26" t="n"/>
+      <c r="F2" s="26" t="n"/>
+      <c r="G2" s="26" t="n"/>
+      <c r="H2" s="26" t="n"/>
+      <c r="I2" s="26" t="n"/>
+      <c r="J2" s="26" t="n"/>
+      <c r="K2" s="27" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="n"/>
+      <c r="B3" s="28" t="n"/>
+      <c r="C3" s="28" t="n"/>
+      <c r="D3" s="28" t="n"/>
+      <c r="E3" s="28" t="n"/>
+      <c r="F3" s="28" t="n"/>
+      <c r="G3" s="28" t="n"/>
+      <c r="H3" s="28" t="n"/>
+      <c r="I3" s="28" t="n"/>
+      <c r="J3" s="28" t="n"/>
+      <c r="K3" s="28" t="n"/>
+    </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Тип</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="29" t="inlineStr">
         <is>
           <t>Раздел ТЗ</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="29" t="inlineStr">
         <is>
           <t>Требование / вопрос</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="29" t="inlineStr">
         <is>
           <t>Где смотреть в UI</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="29" t="inlineStr">
         <is>
           <t>Что проверить</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="29" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="29" t="inlineStr">
         <is>
           <t>Как реализовано сейчас</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="29" t="inlineStr">
         <is>
           <t>Что нужно от backend / данные</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="29" t="inlineStr">
         <is>
           <t>Комментарий / действие</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="29" t="inlineStr">
         <is>
           <t>Комментарии заказчика</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="4" t="n">
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="30" t="inlineStr">
         <is>
           <t>Важно / 1.2</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="30" t="inlineStr">
         <is>
           <t>ИИ не принимает инженерные решения; каждый ответ содержит источник.</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="30" t="inlineStr">
         <is>
           <t>Чат / Проверка</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="30" t="inlineStr">
         <is>
           <t>Проверить, что ответ справочный, а не директивный, и рядом есть «Страница» / «Документ».</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="31" t="inlineStr">
         <is>
           <t>Закрыто на уровне UI</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="30" t="inlineStr">
         <is>
           <t>Ответы оформлены как пояснения для инженера; ссылки на страницу и документ встроены в ответ.</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="30" t="inlineStr">
         <is>
           <t>Backend должен возвращать источники к каждому смысловому пункту ответа.</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="30" t="inlineStr">
         <is>
           <t>Следить, чтобы формулировки не выглядели как автоматическое инженерное решение.</t>
         </is>
       </c>
-      <c r="K5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="7" t="n">
+      <c r="K5" s="30" t="n"/>
+    </row>
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="32" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="32" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="32" t="inlineStr">
         <is>
           <t>Быстрый доступ к НСИ и единая точка поиска по документам.</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="32" t="inlineStr">
         <is>
           <t>Чат / Поиск / Реестр</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="32" t="inlineStr">
         <is>
           <t>Проверить, что инженер может начать с вопроса, поиска или просмотра реестра.</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G6" s="33" t="inlineStr">
         <is>
           <t>Закрыто при наличии backend</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H6" s="32" t="inlineStr">
         <is>
           <t>UI показывает единый вход в базу знаний: чат, поиск, реестр и проверка.</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="I6" s="32" t="inlineStr">
         <is>
           <t>Нужны реальные индексы, RAG-поиск и API с данными документов.</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="J6" s="32" t="inlineStr">
         <is>
           <t>На mock-данных сценарий демонстрируется, фактическая скорость зависит от backend.</t>
         </is>
       </c>
-      <c r="K6" s="8" t="n"/>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="4" t="n">
+      <c r="K6" s="32" t="n"/>
+    </row>
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="30" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Роли пользователей: инженер, администратор знаний, администратор системы.</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Верхняя панель / Навигация / Администрирование</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Выбрать разных пользователей и проверить доступные вкладки.</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>2 / ответ заказчика 05.05.2026</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>Роли пользователей: пользователь и администратор; перед входом нужен отдельный экран авторизации.</t>
+        </is>
+      </c>
+      <c r="E7" s="30" t="inlineStr">
+        <is>
+          <t>Экран входа / Верхняя панель / Навигация / Администрирование</t>
+        </is>
+      </c>
+      <c r="F7" s="30" t="inlineStr">
+        <is>
+          <t>Войти под пользователем и администратором, проверить ФИО, должность, роль и доступные вкладки.</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="inlineStr">
         <is>
           <t>Закрыто на уровне UI</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>В правом верхнем углу показываются ФИО, должность и роль; доступные вкладки меняются по роли.</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Backend должен отдавать профиль пользователя, роль и права после авторизации.</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>В demo-режиме роли переключаются вручную.</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="n"/>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="7" t="n">
+      <c r="H7" s="30" t="inlineStr">
+        <is>
+          <t>Добавлен отдельный экран входа. После входа показываются ФИО, должность и роль; вкладки фильтруются по роли.</t>
+        </is>
+      </c>
+      <c r="I7" s="30" t="inlineStr">
+        <is>
+          <t>Backend должен отдавать профиль пользователя после авторизации: userId, ФИО, должность, роль, права и доступные вкладки.</t>
+        </is>
+      </c>
+      <c r="J7" s="30" t="inlineStr">
+        <is>
+          <t>В demo-режиме вход выполняется выбором тестового пользователя. Реальный логин/пароль подключается через auth-service.</t>
+        </is>
+      </c>
+      <c r="K7" s="30" t="inlineStr">
+        <is>
+          <t>Заказчик подтвердил: нужен отдельный экран авторизации; роли пока — администратор и пользователь.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="78" customHeight="1">
+      <c r="A8" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="32" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="32" t="inlineStr">
         <is>
           <t>2 / 7.1</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Администрирование пользователей, ролей и настроек.</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="D8" s="32" t="inlineStr">
+        <is>
+          <t>Администрирование пользователей, ролей и прав доступа.</t>
+        </is>
+      </c>
+      <c r="E8" s="32" t="inlineStr">
         <is>
           <t>Администрирование</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="32" t="inlineStr">
         <is>
           <t>Выбрать пользователя, изменить роль, включить/выключить права, нажать «Сохранить изменения».</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="31" t="inlineStr">
         <is>
           <t>Закрыто на уровне UI</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>Вкладка администрирования стала функциональной: выбор пользователя, права чекбоксами, сохранение в UI-state и журнал.</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="inlineStr">
+      <c r="H8" s="32" t="inlineStr">
+        <is>
+          <t>Вкладка администрирования функциональна: выбор пользователя, изменение роли, настройка прав чекбоксами, сохранение в UI-state и запись в административный журнал.</t>
+        </is>
+      </c>
+      <c r="I8" s="32" t="inlineStr">
         <is>
           <t>Нужны API пользователей, ролей, прав и административного журнала.</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="J8" s="32" t="inlineStr">
         <is>
           <t>После перезагрузки mock-изменения не сохраняются, это зона backend.</t>
         </is>
       </c>
-      <c r="K8" s="8" t="n"/>
-    </row>
-    <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="K8" s="32" t="inlineStr">
+        <is>
+          <t>Роли приведены к двум базовым ролям: пользователь и администратор.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="78" customHeight="1">
+      <c r="A9" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="30" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="30" t="inlineStr">
         <is>
           <t>Загрузка и обработка документов НСИ: PDF, сканы, DOC/DOCX, CAD, HTML/XML, API.</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="30" t="inlineStr">
         <is>
           <t>Реестр / Администрирование</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="30" t="inlineStr">
         <is>
           <t>Проверить наличие загрузки, статусов обработки и служебных разделов.</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="33" t="inlineStr">
         <is>
           <t>Закрыто при наличии backend</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="30" t="inlineStr">
         <is>
           <t>В реестре есть загрузка документов, OCR-переобработка, обновление индекса и статусы.</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" s="30" t="inlineStr">
         <is>
           <t>Backend должен принимать файлы, запускать pipeline обработки и возвращать статусы.</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J9" s="30" t="inlineStr">
         <is>
           <t>CAD/API-интеграции в UI обозначены на уровне сценария, не выполняются без backend.</t>
         </is>
       </c>
-      <c r="K9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="7" t="n">
+      <c r="K9" s="30" t="n"/>
+    </row>
+    <row r="10" ht="78" customHeight="1">
+      <c r="A10" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="32" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="32" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="32" t="inlineStr">
         <is>
           <t>OCR и извлечение текста, таблиц, изображений; fallback OCR.</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="32" t="inlineStr">
         <is>
           <t>Реестр / QA / Администрирование</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="32" t="inlineStr">
         <is>
           <t>Проверить OCR-статусы, проблемные документы и журналы обработки.</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G10" s="33" t="inlineStr">
         <is>
           <t>Закрыто при наличии backend</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="H10" s="32" t="inlineStr">
         <is>
           <t>UI показывает OCR-статусы, качество OCR, очередь/журналы и переобработку.</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
+      <c r="I10" s="32" t="inlineStr">
         <is>
           <t>OCR выполняется backend/pipeline; UI только показывает результат и управляет запуском.</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="J10" s="32" t="inlineStr">
         <is>
           <t>Нужны реальные статусы OCR и ссылки на артефакты распознавания.</t>
         </is>
       </c>
-      <c r="K10" s="8" t="n"/>
-    </row>
-    <row r="11" ht="58" customHeight="1">
-      <c r="A11" s="4" t="n">
+      <c r="K10" s="32" t="n"/>
+    </row>
+    <row r="11" ht="78" customHeight="1">
+      <c r="A11" s="30" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="30" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="30" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="30" t="inlineStr">
         <is>
           <t>Формирование базы знаний: чанки, embeddings, метаданные, обновление.</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="30" t="inlineStr">
         <is>
           <t>Реестр</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="30" t="inlineStr">
         <is>
           <t>Проверить статусы индексации и кнопку обновления индекса.</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="G11" s="33" t="inlineStr">
         <is>
           <t>Закрыто при наличии backend</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" s="30" t="inlineStr">
         <is>
           <t>Реестр показывает индексацию и действия по обновлению базы знаний.</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I11" s="30" t="inlineStr">
         <is>
           <t>Backend должен хранить метаданные, чанки, embeddings и статус индекса.</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="J11" s="30" t="inlineStr">
         <is>
           <t>UI не создает embeddings сам, это правильно для frontend.</t>
         </is>
       </c>
-      <c r="K11" s="5" t="n"/>
-    </row>
-    <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="7" t="n">
+      <c r="K11" s="30" t="n"/>
+    </row>
+    <row r="12" ht="78" customHeight="1">
+      <c r="A12" s="32" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="32" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="32" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="32" t="inlineStr">
         <is>
           <t>RAG-поиск: ответ, документы, фрагменты источников.</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="32" t="inlineStr">
         <is>
           <t>Чат / Поиск</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="32" t="inlineStr">
         <is>
           <t>Задать вопрос и проверить нумерованный ответ со ссылками на страницу и документ.</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="G12" s="33" t="inlineStr">
         <is>
           <t>Закрыто при наличии backend</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="H12" s="32" t="inlineStr">
         <is>
           <t>Чат выводит нумерованные пункты, под каждым есть «Страница» и «Документ»; поиск показывает фрагменты и релевантность.</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
+      <c r="I12" s="32" t="inlineStr">
         <is>
           <t>Backend должен возвращать answer items, citations, page/document preview URL или ID.</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr">
+      <c r="J12" s="32" t="inlineStr">
         <is>
           <t>Сейчас данные mock, но структура UI готова к API.</t>
         </is>
       </c>
-      <c r="K12" s="8" t="n"/>
-    </row>
-    <row r="13" ht="58" customHeight="1">
-      <c r="A13" s="4" t="n">
+      <c r="K12" s="32" t="n"/>
+    </row>
+    <row r="13" ht="78" customHeight="1">
+      <c r="A13" s="30" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="30" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="30" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Диалоговый режим: уточняющие вопросы и контекст диалога.</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Чат</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Проверить, как UI показывает продолжение диалога и возможное уточнение.</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="inlineStr">
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>Диалоговый режим: контекст диалога, уточняющие вопросы и поиск по текущему чату.</t>
+        </is>
+      </c>
+      <c r="E13" s="30" t="inlineStr">
+        <is>
+          <t>Чат / История</t>
+        </is>
+      </c>
+      <c r="F13" s="30" t="inlineStr">
+        <is>
+          <t>Проверить поиск по текущему чату в нижней панели и возможность продолжить выбранный диалог из истории.</t>
+        </is>
+      </c>
+      <c r="G13" s="34" t="inlineStr">
         <is>
           <t>Частично закрыто</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Диалоговый сценарий и история сообщений есть; отдельный реальный сценарий уточнений зависит от ответа backend.</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>Нужен признак `needsClarification` и текст уточняющего вопроса.</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>Стоит согласовать формат уточняющего ответа.</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="n"/>
-    </row>
-    <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="7" t="n">
+      <c r="H13" s="30" t="inlineStr">
+        <is>
+          <t>В чате добавлен компактный поиск по активной беседе в нижней рабочей панели рядом с полем вопроса. Из истории можно открыть диалог и продолжить его на вкладке «Чат».</t>
+        </is>
+      </c>
+      <c r="I13" s="30" t="inlineStr">
+        <is>
+          <t>Backend должен хранить sessionId, сообщения, источники, статусы ответов и возвращать `needs_clarification`, если нужен дополнительный контекст.</t>
+        </is>
+      </c>
+      <c r="J13" s="30" t="inlineStr">
+        <is>
+          <t>Сценарий уточняющих вопросов пока демонстрируется структурой статусов; нужна реальная логика backend.</t>
+        </is>
+      </c>
+      <c r="K13" s="30" t="inlineStr">
+        <is>
+          <t>Заказчик отметил важность разных срезов истории и поиска по чатам для статистики и частых вопросов.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="78" customHeight="1">
+      <c r="A14" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="32" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="32" t="inlineStr">
         <is>
           <t>3.6</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="32" t="inlineStr">
         <is>
           <t>Проверка проектных решений на соответствие НСИ; статусы OK/WARNING/ERROR.</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="32" t="inlineStr">
         <is>
           <t>Проверка</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="32" t="inlineStr">
         <is>
           <t>Выбрать документы, запустить проверку, открыть страницу/документ и выгрузить Excel.</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="G14" s="33" t="inlineStr">
         <is>
           <t>Закрыто при наличии backend</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="H14" s="32" t="inlineStr">
         <is>
           <t>Вкладка проверяет проектное решение против требования НСИ, показывает проект, раздел, параметр, статус и ссылки.</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr">
+      <c r="I14" s="32" t="inlineStr">
         <is>
           <t>Backend должен возвращать результаты сопоставления и источник требования НСИ.</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr">
+      <c r="J14" s="32" t="inlineStr">
         <is>
           <t>UI готов для выборочной и пакетной проверки.</t>
         </is>
       </c>
-      <c r="K14" s="8" t="n"/>
-    </row>
-    <row r="15" ht="58" customHeight="1">
-      <c r="A15" s="4" t="n">
+      <c r="K14" s="32" t="n"/>
+    </row>
+    <row r="15" ht="78" customHeight="1">
+      <c r="A15" s="30" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="30" t="inlineStr">
         <is>
           <t>3.7</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="30" t="inlineStr">
         <is>
           <t>Рекомендательная система: конфликты, альтернативы, смежные системы.</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="30" t="inlineStr">
         <is>
           <t>Чат / Проверка / QA</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="30" t="inlineStr">
         <is>
           <t>Проверить, есть ли понятный вывод конфликта или альтернативы.</t>
         </is>
       </c>
-      <c r="G15" s="10" t="inlineStr">
+      <c r="G15" s="34" t="inlineStr">
         <is>
           <t>Частично закрыто</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="30" t="inlineStr">
         <is>
           <t>В UI есть статусы предупреждений и проверок, но отдельного блока рекомендаций пока нет.</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="I15" s="30" t="inlineStr">
         <is>
           <t>Backend должен выявлять конфликты и отдавать альтернативы/пояснения.</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="J15" s="30" t="inlineStr">
         <is>
           <t>Нужно решить, нужен ли отдельный экран или достаточно блока в чате/проверке.</t>
         </is>
       </c>
-      <c r="K15" s="5" t="n"/>
-    </row>
-    <row r="16" ht="58" customHeight="1">
-      <c r="A16" s="7" t="n">
+      <c r="K15" s="30" t="n"/>
+    </row>
+    <row r="16" ht="78" customHeight="1">
+      <c r="A16" s="32" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="32" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>3.8</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="C16" s="32" t="inlineStr">
+        <is>
+          <t>3.8 / ответ заказчика 05.05.2026</t>
+        </is>
+      </c>
+      <c r="D16" s="32" t="inlineStr">
         <is>
           <t>Расчетный модуль: перерасчет параметров по методикам НСИ.</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Нет отдельного экрана</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Проверить наличие формы расчета параметров и результата расчета.</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>Не закрыто</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>Отдельного расчетного модуля в текущем UI нет.</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>Нужен backend расчетов и согласованная форма входных параметров.</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>Решить, входит ли расчетный модуль в MVP или следующий этап.</t>
-        </is>
-      </c>
-      <c r="K16" s="8" t="n"/>
-    </row>
-    <row r="17" ht="58" customHeight="1">
-      <c r="A17" s="4" t="n">
+      <c r="E16" s="32" t="inlineStr">
+        <is>
+          <t>Не входит в текущий MVP</t>
+        </is>
+      </c>
+      <c r="F16" s="32" t="inlineStr">
+        <is>
+          <t>Проверить, что расчетный модуль не заявлен как готовая функция текущего MVP.</t>
+        </is>
+      </c>
+      <c r="G16" s="35" t="inlineStr">
+        <is>
+          <t>Исключено из MVP</t>
+        </is>
+      </c>
+      <c r="H16" s="32" t="inlineStr">
+        <is>
+          <t>Отдельного расчетного модуля в текущем UI нет; это соответствует ответу заказчика по текущему объему MVP.</t>
+        </is>
+      </c>
+      <c r="I16" s="32" t="inlineStr">
+        <is>
+          <t>Backend расчетов на текущем этапе не требуется. Если модуль вернется в объем, нужен отдельный API и форма входных параметров.</t>
+        </is>
+      </c>
+      <c r="J16" s="32" t="inlineStr">
+        <is>
+          <t>Не закладывать в демонстрацию как обязательный сценарий текущей версии.</t>
+        </is>
+      </c>
+      <c r="K16" s="32" t="inlineStr">
+        <is>
+          <t>Заказчик ответил: расчетный модуль пока исключен.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="78" customHeight="1">
+      <c r="A17" s="30" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="30" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>3.9</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>История: запрос, ответ, пользователь, источники, поиск, аналитика, экспорт.</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>История</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>Проверить фильтры, таблицу истории и экспорт текущей выборки.</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>3.9 / ответ заказчика 05.05.2026</t>
+        </is>
+      </c>
+      <c r="D17" s="30" t="inlineStr">
+        <is>
+          <t>История диалогов: запросы, ответы, пользователь, источники, разные срезы, поиск и экспорт.</t>
+        </is>
+      </c>
+      <c r="E17" s="30" t="inlineStr">
+        <is>
+          <t>История / Чат</t>
+        </is>
+      </c>
+      <c r="F17" s="30" t="inlineStr">
+        <is>
+          <t>Проверить компактные фильтры по пользователю, проекту, теме, статусу, поиск по тексту, раскрытие диалога внутри таблицы, продолжение чата и экспорт.</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="inlineStr">
         <is>
           <t>Закрыто при наличии backend</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>В истории есть пользователь, статус, запрос/ответ, источники, фильтры и экспорт.</t>
-        </is>
-      </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>Backend должен хранить события и отдавать историю с фильтрами/пагинацией.</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>Экспорт работает на текущих demo-данных.</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="n"/>
-    </row>
-    <row r="18" ht="58" customHeight="1">
-      <c r="A18" s="7" t="n">
+      <c r="H17" s="30" t="inlineStr">
+        <is>
+          <t>История дополнена срезами: пользователь, проект, тема, сессия. По клику строка раскрывает диалог прямо внутри таблицы, есть кнопка «Продолжить чат» и экспорт текущей выборки.</t>
+        </is>
+      </c>
+      <c r="I17" s="30" t="inlineStr">
+        <is>
+          <t>Backend должен хранить диалоги с sessionId, проектом, темой, пользователем, сообщениями, источниками и поддерживать фильтры/пагинацию/экспорт. Пользователь должен получать свои диалоги, администратор — все или фильтрованные диалоги.</t>
+        </is>
+      </c>
+      <c r="J17" s="30" t="inlineStr">
+        <is>
+          <t>Правило доступа фиксируем простое: пользователь видит свои чаты, администратор видит все чаты для QA, статистики и анализа частых вопросов.</t>
+        </is>
+      </c>
+      <c r="K17" s="30" t="inlineStr">
+        <is>
+          <t>Заказчик подтвердил потребность в разных срезах истории; конкретная организация — технический вопрос.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="78" customHeight="1">
+      <c r="A18" s="32" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="32" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="32" t="inlineStr">
         <is>
           <t>3.10</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="32" t="inlineStr">
         <is>
           <t>Интеграция с ИС «Меридиан»: получение данных, запись результатов, история.</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E18" s="32" t="inlineStr">
         <is>
           <t>README / будущий backend</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F18" s="32" t="inlineStr">
         <is>
           <t>Проверить, есть ли отдельный статус Meridian или экран интеграции.</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G18" s="34" t="inlineStr">
         <is>
           <t>Частично закрыто</t>
         </is>
       </c>
-      <c r="H18" s="8" t="inlineStr">
+      <c r="H18" s="32" t="inlineStr">
         <is>
           <t>UI готов работать через HTTP API, но отдельной индикации Meridian пока нет.</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr">
+      <c r="I18" s="32" t="inlineStr">
         <is>
           <t>Нужны endpoints интеграции и статусы синхронизации.</t>
         </is>
       </c>
-      <c r="J18" s="8" t="inlineStr">
+      <c r="J18" s="32" t="inlineStr">
         <is>
           <t>Уточнить, надо ли показывать Meridian явно в UI.</t>
         </is>
       </c>
-      <c r="K18" s="8" t="n"/>
-    </row>
-    <row r="19" ht="58" customHeight="1">
-      <c r="A19" s="4" t="n">
+      <c r="K18" s="32" t="n"/>
+    </row>
+    <row r="19" ht="78" customHeight="1">
+      <c r="A19" s="30" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="30" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="30" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="30" t="inlineStr">
         <is>
           <t>Нефункциональные требования: время ответа, OCR, точность, нагрузка, доступность, безопасность.</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="30" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" s="30" t="inlineStr">
         <is>
           <t>Проверить, что метрики читаются и связаны с критериями приемки.</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr">
+      <c r="G19" s="34" t="inlineStr">
         <is>
           <t>Частично закрыто</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H19" s="30" t="inlineStr">
         <is>
           <t>QA-вкладка показывает скорость, OCR, точность, источники и журнал проверки.</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="I19" s="30" t="inlineStr">
         <is>
           <t>Backend/мониторинг должны отдавать реальные значения метрик.</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="J19" s="30" t="inlineStr">
         <is>
           <t>Безопасность и доступность не проверяются на frontend mock-уровне.</t>
         </is>
       </c>
-      <c r="K19" s="5" t="n"/>
-    </row>
-    <row r="20" ht="58" customHeight="1">
-      <c r="A20" s="7" t="n">
+      <c r="K19" s="30" t="n"/>
+    </row>
+    <row r="20" ht="78" customHeight="1">
+      <c r="A20" s="32" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="32" t="inlineStr">
         <is>
           <t>ТЗ</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="32" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="32" t="inlineStr">
         <is>
           <t>Frontend: React, TypeScript, UI Ant Design / shadcn.</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E20" s="32" t="inlineStr">
         <is>
           <t>Код frontend</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F20" s="32" t="inlineStr">
         <is>
           <t>Проверить стек проекта.</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="G20" s="34" t="inlineStr">
+        <is>
+          <t>Закрыто на уровне команды</t>
+        </is>
+      </c>
+      <c r="H20" s="32" t="inlineStr">
+        <is>
+          <t>Текущая UI V1 реализована на React + TypeScript + Vite + MUI. Выбор библиотеки остается техническим решением команды.</t>
+        </is>
+      </c>
+      <c r="I20" s="32" t="inlineStr">
+        <is>
+          <t>Backend не влияет; нужно решение команды/заказчика по допустимости MUI.</t>
+        </is>
+      </c>
+      <c r="J20" s="32" t="inlineStr">
+        <is>
+          <t>Не выносить выбор UI-библиотеки на заказчика как функциональное требование.</t>
+        </is>
+      </c>
+      <c r="K20" s="32" t="inlineStr">
+        <is>
+          <t>Заказчик ответил: UI-библиотеки — технический вопрос, заказчик его не решает.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="78" customHeight="1">
+      <c r="A21" s="30" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>ТЗ</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D21" s="30" t="inlineStr">
+        <is>
+          <t>Архитектура: Frontend → Backend API → RAG/Vector DB/LLM.</t>
+        </is>
+      </c>
+      <c r="E21" s="30" t="inlineStr">
+        <is>
+          <t>README / frontend/src/utils/http.ts</t>
+        </is>
+      </c>
+      <c r="F21" s="30" t="inlineStr">
+        <is>
+          <t>Проверить, что UI отделен от backend и работает через HTTP-вызовы.</t>
+        </is>
+      </c>
+      <c r="G21" s="33" t="inlineStr">
+        <is>
+          <t>Закрыто при наличии backend</t>
+        </is>
+      </c>
+      <c r="H21" s="30" t="inlineStr">
+        <is>
+          <t>Frontend не содержит backend-логики; API-контур описан в README и utils/http.ts.</t>
+        </is>
+      </c>
+      <c r="I21" s="30" t="inlineStr">
+        <is>
+          <t>Нужны реальные endpoints, OpenAPI и единые DTO.</t>
+        </is>
+      </c>
+      <c r="J21" s="30" t="inlineStr">
+        <is>
+          <t>Хорошая база для подключения backend без переделки экранов.</t>
+        </is>
+      </c>
+      <c r="K21" s="30" t="n"/>
+    </row>
+    <row r="22" ht="78" customHeight="1">
+      <c r="A22" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="32" t="inlineStr">
+        <is>
+          <t>ТЗ</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="D22" s="32" t="inlineStr">
+        <is>
+          <t>Основные экраны: авторизация, ввод запроса, ответ с источниками, диалог, история, администрирование.</t>
+        </is>
+      </c>
+      <c r="E22" s="32" t="inlineStr">
+        <is>
+          <t>Все вкладки</t>
+        </is>
+      </c>
+      <c r="F22" s="32" t="inlineStr">
+        <is>
+          <t>Проверить наличие всех основных экранов.</t>
+        </is>
+      </c>
+      <c r="G22" s="31" t="inlineStr">
+        <is>
+          <t>Закрыто на уровне UI</t>
+        </is>
+      </c>
+      <c r="H22" s="32" t="inlineStr">
+        <is>
+          <t>Есть экран входа, чат с поиском по текущей беседе, поиск, реестр, проверка, история диалогов с раскрытием строки, QA и администрирование.</t>
+        </is>
+      </c>
+      <c r="I22" s="32" t="inlineStr">
+        <is>
+          <t>Backend нужен для наполнения реальными данными.</t>
+        </is>
+      </c>
+      <c r="J22" s="32" t="inlineStr">
+        <is>
+          <t>Экран администрирования добавлен и работает в demo-режиме.</t>
+        </is>
+      </c>
+      <c r="K22" s="32" t="inlineStr">
+        <is>
+          <t>Добавление экрана авторизации соответствует ответу заказчика.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="78" customHeight="1">
+      <c r="A23" s="30" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>ТЗ</t>
+        </is>
+      </c>
+      <c r="C23" s="30" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="D23" s="30" t="inlineStr">
+        <is>
+          <t>UX: one-shot, прозрачность источников, управляемость пользователем.</t>
+        </is>
+      </c>
+      <c r="E23" s="30" t="inlineStr">
+        <is>
+          <t>Чат / Превью / Фокус-режим</t>
+        </is>
+      </c>
+      <c r="F23" s="30" t="inlineStr">
+        <is>
+          <t>Проверить, видно ли ответ, источники и действия без лишнего скролла.</t>
+        </is>
+      </c>
+      <c r="G23" s="31" t="inlineStr">
+        <is>
+          <t>Закрыто на уровне UI</t>
+        </is>
+      </c>
+      <c r="H23" s="30" t="inlineStr">
+        <is>
+          <t>Ответы в чате читаются как пункты; страница и документ открываются справа; есть поиск по активному чату и фокус-режим.</t>
+        </is>
+      </c>
+      <c r="I23" s="30" t="inlineStr">
+        <is>
+          <t>Backend должен возвращать корректные источники и статусы.</t>
+        </is>
+      </c>
+      <c r="J23" s="30" t="inlineStr">
+        <is>
+          <t>Текущий UX ориентирован на инженерный сценарий.</t>
+        </is>
+      </c>
+      <c r="K23" s="30" t="n"/>
+    </row>
+    <row r="24" ht="78" customHeight="1">
+      <c r="A24" s="32" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="32" t="inlineStr">
+        <is>
+          <t>ТЗ</t>
+        </is>
+      </c>
+      <c r="C24" s="32" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D24" s="32" t="inlineStr">
+        <is>
+          <t>Критерии приемки: точность ≥85%, скорость ≤30 сек, OCR ≥80%, источники 100%.</t>
+        </is>
+      </c>
+      <c r="E24" s="32" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="F24" s="32" t="inlineStr">
+        <is>
+          <t>Проверить, что эти показатели представлены в интерфейсе.</t>
+        </is>
+      </c>
+      <c r="G24" s="33" t="inlineStr">
+        <is>
+          <t>Закрыто при наличии backend</t>
+        </is>
+      </c>
+      <c r="H24" s="32" t="inlineStr">
+        <is>
+          <t>QA показывает метрики, статусы и журнал проверки; UI готов отражать критерии приемки.</t>
+        </is>
+      </c>
+      <c r="I24" s="32" t="inlineStr">
+        <is>
+          <t>Нужны тестовые прогоны и реальные метрики от backend/QA pipeline.</t>
+        </is>
+      </c>
+      <c r="J24" s="32" t="inlineStr">
+        <is>
+          <t>Цифры сейчас демонстрационные.</t>
+        </is>
+      </c>
+      <c r="K24" s="32" t="n"/>
+    </row>
+    <row r="25" ht="78" customHeight="1">
+      <c r="A25" s="30" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>ТЗ</t>
+        </is>
+      </c>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D25" s="30" t="inlineStr">
+        <is>
+          <t>Поставка: Git, docker-compose, README, OpenAPI, тесты, deploy.</t>
+        </is>
+      </c>
+      <c r="E25" s="30" t="inlineStr">
+        <is>
+          <t>README / frontend</t>
+        </is>
+      </c>
+      <c r="F25" s="30" t="inlineStr">
+        <is>
+          <t>Проверить запуск через Docker и наличие инструкции.</t>
+        </is>
+      </c>
+      <c r="G25" s="34" t="inlineStr">
         <is>
           <t>Частично закрыто</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>Реализовано на React + TypeScript + Vite + MUI.</t>
-        </is>
-      </c>
-      <c r="I20" s="8" t="inlineStr">
-        <is>
-          <t>Backend не влияет; нужно решение команды/заказчика по допустимости MUI.</t>
-        </is>
-      </c>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>Если строго требуется Ant Design/shadcn, потребуется миграция UI-библиотеки.</t>
-        </is>
-      </c>
-      <c r="K20" s="8" t="n"/>
-    </row>
-    <row r="21" ht="58" customHeight="1">
-      <c r="A21" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>ТЗ</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Архитектура: Frontend → Backend API → RAG/Vector DB/LLM.</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>README / frontend/src/utils/http.ts</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>Проверить, что UI отделен от backend и работает через HTTP-вызовы.</t>
-        </is>
-      </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="H25" s="30" t="inlineStr">
+        <is>
+          <t>Есть Dockerfile, docker-compose, README и рабочий frontend-контур.</t>
+        </is>
+      </c>
+      <c r="I25" s="30" t="inlineStr">
+        <is>
+          <t>OpenAPI, интеграционные тесты и полный deploy-контур должны прийти вместе с backend.</t>
+        </is>
+      </c>
+      <c r="J25" s="30" t="inlineStr">
+        <is>
+          <t>Для frontend demo поставка достаточная.</t>
+        </is>
+      </c>
+      <c r="K25" s="30" t="n"/>
+    </row>
+    <row r="26" ht="78" customHeight="1">
+      <c r="A26" s="32" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="32" t="inlineStr">
+        <is>
+          <t>Доп. UI/UX</t>
+        </is>
+      </c>
+      <c r="C26" s="32" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="D26" s="32" t="inlineStr">
+        <is>
+          <t>Фокус-режим для работы без левой панели.</t>
+        </is>
+      </c>
+      <c r="E26" s="32" t="inlineStr">
+        <is>
+          <t>Все вкладки</t>
+        </is>
+      </c>
+      <c r="F26" s="32" t="inlineStr">
+        <is>
+          <t>Нажать «Фокус-режим» на разных вкладках и выйти обратно.</t>
+        </is>
+      </c>
+      <c r="G26" s="31" t="inlineStr">
+        <is>
+          <t>Закрыто на уровне UI</t>
+        </is>
+      </c>
+      <c r="H26" s="32" t="inlineStr">
+        <is>
+          <t>Фокус-режим доступен на каждой вкладке и скрывает навигацию.</t>
+        </is>
+      </c>
+      <c r="I26" s="32" t="inlineStr">
+        <is>
+          <t>Backend не требуется.</t>
+        </is>
+      </c>
+      <c r="J26" s="32" t="inlineStr">
+        <is>
+          <t>Полезно для демонстрации и работы с таблицами/документами.</t>
+        </is>
+      </c>
+      <c r="K26" s="32" t="n"/>
+    </row>
+    <row r="27" ht="78" customHeight="1">
+      <c r="A27" s="30" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>Доп. UI/UX</t>
+        </is>
+      </c>
+      <c r="C27" s="30" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="D27" s="30" t="inlineStr">
+        <is>
+          <t>Темная и светлая тема интерфейса.</t>
+        </is>
+      </c>
+      <c r="E27" s="30" t="inlineStr">
+        <is>
+          <t>Верхняя панель</t>
+        </is>
+      </c>
+      <c r="F27" s="30" t="inlineStr">
+        <is>
+          <t>Переключить тему и проверить читаемость всех вкладок.</t>
+        </is>
+      </c>
+      <c r="G27" s="31" t="inlineStr">
+        <is>
+          <t>Закрыто на уровне UI</t>
+        </is>
+      </c>
+      <c r="H27" s="30" t="inlineStr">
+        <is>
+          <t>Есть темная и светлая темы, текущая светлая тема приведена к читаемому виду.</t>
+        </is>
+      </c>
+      <c r="I27" s="30" t="inlineStr">
+        <is>
+          <t>Backend не требуется.</t>
+        </is>
+      </c>
+      <c r="J27" s="30" t="inlineStr">
+        <is>
+          <t>Продолжать визуальную полировку после отзывов команды.</t>
+        </is>
+      </c>
+      <c r="K27" s="30" t="n"/>
+    </row>
+    <row r="28" ht="78" customHeight="1">
+      <c r="A28" s="32" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="32" t="inlineStr">
+        <is>
+          <t>Доп. UI/UX</t>
+        </is>
+      </c>
+      <c r="C28" s="32" t="inlineStr">
+        <is>
+          <t>Демо</t>
+        </is>
+      </c>
+      <c r="D28" s="32" t="inlineStr">
+        <is>
+          <t>Видеоинструкция внутри интерфейса.</t>
+        </is>
+      </c>
+      <c r="E28" s="32" t="inlineStr">
+        <is>
+          <t>Верхняя панель</t>
+        </is>
+      </c>
+      <c r="F28" s="32" t="inlineStr">
+        <is>
+          <t>Открыть видеоинструкцию и проверить полноэкранный сценарий.</t>
+        </is>
+      </c>
+      <c r="G28" s="31" t="inlineStr">
+        <is>
+          <t>Закрыто на уровне UI</t>
+        </is>
+      </c>
+      <c r="H28" s="32" t="inlineStr">
+        <is>
+          <t>Есть кнопка видеоинструкции и fullscreen demo-сценарий.</t>
+        </is>
+      </c>
+      <c r="I28" s="32" t="inlineStr">
+        <is>
+          <t>Backend не требуется.</t>
+        </is>
+      </c>
+      <c r="J28" s="32" t="inlineStr">
+        <is>
+          <t>Видео можно обновлять отдельно от кода UI.</t>
+        </is>
+      </c>
+      <c r="K28" s="32" t="n"/>
+    </row>
+    <row r="29" ht="78" customHeight="1">
+      <c r="A29" s="30" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t>ТЗ / QA</t>
+        </is>
+      </c>
+      <c r="C29" s="30" t="inlineStr">
+        <is>
+          <t>4 / 8</t>
+        </is>
+      </c>
+      <c r="D29" s="30" t="inlineStr">
+        <is>
+          <t>Оценка ответов инженерами для QA и улучшения качества.</t>
+        </is>
+      </c>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>Чат / QA</t>
+        </is>
+      </c>
+      <c r="F29" s="30" t="inlineStr">
+        <is>
+          <t>Поставить оценку ответу, добавить комментарий, проверить отражение в QA-логике.</t>
+        </is>
+      </c>
+      <c r="G29" s="33" t="inlineStr">
         <is>
           <t>Закрыто при наличии backend</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>Frontend не содержит backend-логики; API-контур описан в README и utils/http.ts.</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>Нужны реальные endpoints, OpenAPI и единые DTO.</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>Хорошая база для подключения backend без переделки экранов.</t>
-        </is>
-      </c>
-      <c r="K21" s="5" t="n"/>
-    </row>
-    <row r="22" ht="58" customHeight="1">
-      <c r="A22" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>ТЗ</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>7.1</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Основные экраны: ввод запроса, ответ с источниками, диалог, история, администрирование.</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>Все вкладки</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Проверить наличие всех основных экранов.</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>Закрыто на уровне UI</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>Есть чат, поиск, реестр, проверка, история, QA и администрирование.</t>
-        </is>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>Backend нужен для наполнения реальными данными.</t>
-        </is>
-      </c>
-      <c r="J22" s="8" t="inlineStr">
-        <is>
-          <t>Экран администрирования добавлен и работает в demo-режиме.</t>
-        </is>
-      </c>
-      <c r="K22" s="8" t="n"/>
-    </row>
-    <row r="23" ht="58" customHeight="1">
-      <c r="A23" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>ТЗ</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>7.2</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>UX: one-shot, прозрачность источников, управляемость пользователем.</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Чат / Превью / Фокус-режим</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>Проверить, видно ли ответ, источники и действия без лишнего скролла.</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>Закрыто на уровне UI</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>Ответы в чате читаются как пункты; страница и документ открываются справа; есть фокус-режим.</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>Backend должен возвращать корректные источники и статусы.</t>
-        </is>
-      </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>Текущий UX ориентирован на инженерный сценарий.</t>
-        </is>
-      </c>
-      <c r="K23" s="5" t="n"/>
-    </row>
-    <row r="24" ht="58" customHeight="1">
-      <c r="A24" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>ТЗ</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Критерии приемки: точность ≥85%, скорость ≤30 сек, OCR ≥80%, источники 100%.</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>Проверить, что эти показатели представлены в интерфейсе.</t>
-        </is>
-      </c>
-      <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>Закрыто при наличии backend</t>
-        </is>
-      </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>QA показывает метрики, статусы и журнал проверки; UI готов отражать критерии приемки.</t>
-        </is>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Нужны тестовые прогоны и реальные метрики от backend/QA pipeline.</t>
-        </is>
-      </c>
-      <c r="J24" s="8" t="inlineStr">
-        <is>
-          <t>Цифры сейчас демонстрационные.</t>
-        </is>
-      </c>
-      <c r="K24" s="8" t="n"/>
-    </row>
-    <row r="25" ht="58" customHeight="1">
-      <c r="A25" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>ТЗ</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Поставка: Git, docker-compose, README, OpenAPI, тесты, deploy.</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>README / frontend</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>Проверить запуск через Docker и наличие инструкции.</t>
-        </is>
-      </c>
-      <c r="G25" s="10" t="inlineStr">
-        <is>
-          <t>Частично закрыто</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>Есть Dockerfile, docker-compose, README и рабочий frontend-контур.</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>OpenAPI, интеграционные тесты и полный deploy-контур должны прийти вместе с backend.</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>Для frontend demo поставка достаточная.</t>
-        </is>
-      </c>
-      <c r="K25" s="5" t="n"/>
-    </row>
-    <row r="26" ht="58" customHeight="1">
-      <c r="A26" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Доп. UI/UX</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>7.2</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Фокус-режим для работы без левой панели.</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>Все вкладки</t>
-        </is>
-      </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Нажать «Фокус-режим» на разных вкладках и выйти обратно.</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>Закрыто на уровне UI</t>
-        </is>
-      </c>
-      <c r="H26" s="8" t="inlineStr">
-        <is>
-          <t>Фокус-режим доступен на каждой вкладке и скрывает навигацию.</t>
-        </is>
-      </c>
-      <c r="I26" s="8" t="inlineStr">
-        <is>
-          <t>Backend не требуется.</t>
-        </is>
-      </c>
-      <c r="J26" s="8" t="inlineStr">
-        <is>
-          <t>Полезно для демонстрации и работы с таблицами/документами.</t>
-        </is>
-      </c>
-      <c r="K26" s="8" t="n"/>
-    </row>
-    <row r="27" ht="58" customHeight="1">
-      <c r="A27" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Доп. UI/UX</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>7.2</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>Темная и светлая тема интерфейса.</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Верхняя панель</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>Переключить тему и проверить читаемость всех вкладок.</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>Закрыто на уровне UI</t>
-        </is>
-      </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>Есть темная и светлая темы, текущая светлая тема приведена к читаемому виду.</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>Backend не требуется.</t>
-        </is>
-      </c>
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>Продолжать визуальную полировку после отзывов команды.</t>
-        </is>
-      </c>
-      <c r="K27" s="5" t="n"/>
-    </row>
-    <row r="28" ht="58" customHeight="1">
-      <c r="A28" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Доп. UI/UX</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>Демо</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Видеоинструкция внутри интерфейса.</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>Верхняя панель</t>
-        </is>
-      </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>Открыть видеоинструкцию и проверить полноэкранный сценарий.</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>Закрыто на уровне UI</t>
-        </is>
-      </c>
-      <c r="H28" s="8" t="inlineStr">
-        <is>
-          <t>Есть кнопка видеоинструкции и fullscreen demo-сценарий.</t>
-        </is>
-      </c>
-      <c r="I28" s="8" t="inlineStr">
-        <is>
-          <t>Backend не требуется.</t>
-        </is>
-      </c>
-      <c r="J28" s="8" t="inlineStr">
-        <is>
-          <t>Видео можно обновлять отдельно от кода UI.</t>
-        </is>
-      </c>
-      <c r="K28" s="8" t="n"/>
-    </row>
-    <row r="29" ht="58" customHeight="1">
-      <c r="A29" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>ТЗ / QA</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>4 / 8</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Оценка ответов инженерами для QA и улучшения качества.</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Чат / QA</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>Поставить оценку ответу, добавить комментарий, проверить отражение в QA-логике.</t>
-        </is>
-      </c>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>Закрыто при наличии backend</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="H29" s="30" t="inlineStr">
         <is>
           <t>Feedback-компонент есть; QA-вкладка показывает оценку ответов ассистента.</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>Нужно сохранять feedback в backend и учитывать в метриках качества/тестовых наборах.</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
+      <c r="I29" s="30" t="inlineStr">
+        <is>
+          <t>Нужно сохранять feedback в backend и учитывать в QA-метриках, тестовых наборах, статистике частых вопросов и улучшении формулировок ответов.</t>
+        </is>
+      </c>
+      <c r="J29" s="30" t="inlineStr">
         <is>
           <t>Это важный контур для будущей приемки и улучшения ответов.</t>
         </is>
       </c>
-      <c r="K29" s="5" t="n"/>
+      <c r="K29" s="30" t="inlineStr">
+        <is>
+          <t>Поиск по чатам и оценки инженеров важны для статистики и ответов на частые вопросы.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:K29"/>
@@ -2101,7 +2202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2110,160 +2211,219 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>Сводка по текущей версии UI</t>
         </is>
       </c>
-      <c r="B1" s="19" t="n"/>
-      <c r="C1" s="19" t="n"/>
-      <c r="D1" s="19" t="n"/>
-      <c r="E1" s="20" t="n"/>
+      <c r="B1" s="24" t="n"/>
+      <c r="C1" s="24" t="n"/>
+      <c r="D1" s="24" t="n"/>
+      <c r="E1" s="25" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="n"/>
+      <c r="B2" s="28" t="n"/>
+      <c r="C2" s="28" t="n"/>
+      <c r="D2" s="28" t="n"/>
+      <c r="E2" s="28" t="n"/>
     </row>
     <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="36" t="inlineStr">
         <is>
           <t>Показатель</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="36" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="36" t="inlineStr">
         <is>
           <t>Комментарий</t>
         </is>
       </c>
+      <c r="D3" s="28" t="n"/>
+      <c r="E3" s="28" t="n"/>
     </row>
     <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="37" t="inlineStr">
         <is>
           <t>Проверяемая версия</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>UI v1 / frontend</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>Последняя локальная версия с ролями, администрированием и светлой/темной темой.</t>
-        </is>
-      </c>
+      <c r="B4" s="37" t="inlineStr">
+        <is>
+          <t>UI v1 / frontend / 2026-05-05</t>
+        </is>
+      </c>
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>Последняя локальная версия с экраном входа, двумя ролями, историей диалогов, поиском по чатам, администрированием и светлой/темной темой.</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="n"/>
+      <c r="E4" s="28" t="n"/>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="37" t="inlineStr">
         <is>
           <t>Основание</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="37" t="inlineStr">
         <is>
           <t>ТЗ нейроассистента ПКБ</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="37" t="inlineStr">
         <is>
           <t>Использованы разделы 1-8 и 11, а также UI/UX требования.</t>
         </is>
       </c>
+      <c r="D5" s="28" t="n"/>
+      <c r="E5" s="28" t="n"/>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>Главный вывод</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="37" t="inlineStr">
         <is>
           <t>Основной инженерный сценарий закрыт на уровне UI</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>Чат, источники, поиск, проверка, история, QA и администрирование готовы как frontend-контур.</t>
-        </is>
-      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>Чат, источники, поиск, проверка, история диалогов, QA, авторизация и администрирование готовы как frontend-контур.</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="n"/>
+      <c r="E6" s="28" t="n"/>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t>Главный риск</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="37" t="inlineStr">
         <is>
           <t>Нет реального backend в этой поставке</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>Фактическая точность, скорость, OCR и сохранение данных подтверждаются только после интеграции.</t>
-        </is>
-      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>Фактическая точность, скорость, OCR, сохранение истории и права доступа подтверждаются только после интеграции backend.</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="n"/>
+      <c r="E7" s="28" t="n"/>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="37" t="inlineStr">
         <is>
           <t>Статус: Закрыто на уровне UI</t>
         </is>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="38" t="n">
         <v>8</v>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="37" t="inlineStr">
         <is>
           <t>Количество пунктов с таким статусом.</t>
         </is>
       </c>
+      <c r="D8" s="28" t="n"/>
+      <c r="E8" s="28" t="n"/>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>Статус: Закрыто при наличии backend</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="39" t="n">
         <v>10</v>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="37" t="inlineStr">
         <is>
           <t>Количество пунктов с таким статусом.</t>
         </is>
       </c>
+      <c r="D9" s="28" t="n"/>
+      <c r="E9" s="28" t="n"/>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>Статус: Частично закрыто</t>
         </is>
       </c>
-      <c r="B10" s="17" t="n">
-        <v>6</v>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="B10" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
         <is>
           <t>Количество пунктов с таким статусом.</t>
         </is>
       </c>
+      <c r="D10" s="28" t="n"/>
+      <c r="E10" s="28" t="n"/>
     </row>
     <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t>Статус: Не закрыто</t>
         </is>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>Количество пунктов с таким статусом.</t>
+        </is>
+      </c>
+      <c r="D11" s="28" t="n"/>
+      <c r="E11" s="28" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>Статус: Исключено из MVP</t>
+        </is>
+      </c>
+      <c r="B12" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>Количество пунктов с таким статусом.</t>
-        </is>
-      </c>
+      <c r="C12" s="28" t="inlineStr">
+        <is>
+          <t>Пункт не входит в актуальный объем MVP по ответу заказчика.</t>
+        </is>
+      </c>
+      <c r="D12" s="28" t="n"/>
+      <c r="E12" s="28" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>Статус: Закрыто на уровне команды</t>
+        </is>
+      </c>
+      <c r="B13" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="28" t="inlineStr">
+        <is>
+          <t>Технический выбор команды, не требующий решения заказчика.</t>
+        </is>
+      </c>
+      <c r="D13" s="28" t="n"/>
+      <c r="E13" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2288,99 +2448,110 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>Как пользоваться чек-листом</t>
         </is>
       </c>
-      <c r="B1" s="19" t="n"/>
-      <c r="C1" s="19" t="n"/>
-      <c r="D1" s="20" t="n"/>
+      <c r="B1" s="24" t="n"/>
+      <c r="C1" s="24" t="n"/>
+      <c r="D1" s="25" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="n"/>
+      <c r="B2" s="28" t="n"/>
+      <c r="C2" s="28" t="n"/>
+      <c r="D2" s="28" t="n"/>
     </row>
     <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="36" t="inlineStr">
         <is>
           <t>Поле</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="36" t="inlineStr">
         <is>
           <t>Что писать / как читать</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="36" t="inlineStr">
         <is>
           <t>Пример</t>
         </is>
       </c>
+      <c r="D3" s="28" t="n"/>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="37" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="37" t="inlineStr">
         <is>
           <t>Итог по пункту. Если написано «при наличии backend», значит UI готов, но нужны реальные API и данные.</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="37" t="inlineStr">
         <is>
           <t>Закрыто при наличии backend</t>
         </is>
       </c>
+      <c r="D4" s="28" t="n"/>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="37" t="inlineStr">
         <is>
           <t>Как реализовано сейчас</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="37" t="inlineStr">
         <is>
           <t>Что уже видно или можно проверить в интерфейсе.</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="37" t="inlineStr">
         <is>
           <t>Ответ содержит ссылки «Страница» и «Документ».</t>
         </is>
       </c>
+      <c r="D5" s="28" t="n"/>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>Что нужно от backend / данные</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="37" t="inlineStr">
         <is>
           <t>Какие реальные данные, endpoint или сохранение нужны для production.</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="37" t="inlineStr">
         <is>
           <t>POST /chat должен вернуть citations.</t>
         </is>
       </c>
+      <c r="D6" s="28" t="n"/>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t>Комментарий / действие</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="37" t="inlineStr">
         <is>
           <t>Что уточнить, проверить или доделать дальше.</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="37" t="inlineStr">
         <is>
           <t>Уточнить формат ответа без данных.</t>
         </is>
       </c>
+      <c r="D7" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>